<commit_message>
Changed meta regresssion base
</commit_message>
<xml_diff>
--- a/analysis/Fcheck.xlsx
+++ b/analysis/Fcheck.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tarun\Documents\GitHub\appliances_interventions\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6FAEDBED-E3F3-4484-B65D-AEC76730F630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5724B8B4-571D-4E41-8C60-5A4902D271D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E0D855C0-9398-4A35-9BC6-9F9D377BCE00}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{8F85E8AE-89C1-44AE-A407-F7B5B53EA649}"/>
   </bookViews>
   <sheets>
     <sheet name="Fcheck" sheetId="1" r:id="rId1"/>
@@ -58,28 +58,28 @@
     <t>subsidy</t>
   </si>
   <si>
-    <t>applianceClothes_Dryer</t>
-  </si>
-  <si>
-    <t>applianceDishwasher</t>
-  </si>
-  <si>
-    <t>applianceHeat_Pump</t>
-  </si>
-  <si>
-    <t>applianceLighting</t>
-  </si>
-  <si>
-    <t>applianceRefrigerator</t>
-  </si>
-  <si>
-    <t>applianceTV</t>
-  </si>
-  <si>
-    <t>applianceWashing_Machine</t>
-  </si>
-  <si>
-    <t>applianceWater_Heater</t>
+    <t>appliance1Air-Conditioner</t>
+  </si>
+  <si>
+    <t>appliance1Clothes_Dryer</t>
+  </si>
+  <si>
+    <t>appliance1Dishwasher</t>
+  </si>
+  <si>
+    <t>appliance1Heat_Pump</t>
+  </si>
+  <si>
+    <t>appliance1Lighting</t>
+  </si>
+  <si>
+    <t>appliance1TV</t>
+  </si>
+  <si>
+    <t>appliance1Washing_Machine</t>
+  </si>
+  <si>
+    <t>appliance1Water_Heater</t>
   </si>
   <si>
     <t>incentive_follow_throughself-reported_behavior</t>
@@ -91,10 +91,10 @@
     <t>reportingBiasesprobably_yes</t>
   </si>
   <si>
-    <t>participant_typehomeowners</t>
-  </si>
-  <si>
-    <t>participant_typeunspecified</t>
+    <t>participant_type1homeowners</t>
+  </si>
+  <si>
+    <t>participant_type1unspecified</t>
   </si>
   <si>
     <t>outOfSampleBiasprobably_yes</t>
@@ -634,7 +634,18 @@
     <cellStyle name="Total" xfId="18" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="15" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -963,63 +974,64 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EED73D99-311D-4B49-B7B2-7922E8C44717}">
-  <dimension ref="A1:G21"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90910AB3-ABE6-4911-8C78-C9AB78D0F6C2}">
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="40.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="40.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.6328125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.6328125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C2" s="1">
-        <v>-0.23195876184525999</v>
+        <v>-9.1555865069096895E-2</v>
       </c>
       <c r="D2" s="1">
-        <v>0.126049883661109</v>
+        <v>9.3859846077325004E-2</v>
       </c>
       <c r="E2" s="1">
-        <v>-1.8402140097875199</v>
+        <v>-0.97545296413196703</v>
       </c>
       <c r="F2" s="1">
         <v>48</v>
       </c>
       <c r="G2" s="1">
-        <v>7.1923964390541703E-2</v>
+        <v>0.33422620028866201</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -1029,53 +1041,53 @@
         <v>2.4868891546873599</v>
       </c>
       <c r="D3" s="1">
-        <v>0.36716032223653</v>
+        <v>0.367160322236531</v>
       </c>
       <c r="E3" s="1">
-        <v>6.7733058396361097</v>
+        <v>6.7733058396360901</v>
       </c>
       <c r="F3" s="1">
         <v>48</v>
       </c>
       <c r="G3" s="1">
-        <v>1.6374197954203299E-8</v>
+        <v>1.6374197954204299E-8</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C4" s="1">
-        <v>8.1075539590060707E-3</v>
+        <v>8.1075539590059805E-3</v>
       </c>
       <c r="D4" s="1">
-        <v>5.0957986531035303E-2</v>
+        <v>5.09579865310354E-2</v>
       </c>
       <c r="E4" s="1">
-        <v>0.15910271403812801</v>
+        <v>0.15910271403812601</v>
       </c>
       <c r="F4" s="1">
         <v>48</v>
       </c>
       <c r="G4" s="1">
-        <v>0.87425551696909398</v>
+        <v>0.87425551696909598</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="1">
-        <v>-7.1316269558089104E-2</v>
+        <v>-7.1316269558088993E-2</v>
       </c>
       <c r="D5" s="1">
-        <v>4.7493625032537901E-2</v>
+        <v>4.7493625032537998E-2</v>
       </c>
       <c r="E5" s="1">
         <v>-1.50159667764316</v>
@@ -1084,11 +1096,11 @@
         <v>48</v>
       </c>
       <c r="G5" s="1">
-        <v>0.139751649411231</v>
+        <v>0.139751649411232</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -1111,14 +1123,14 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="1">
-        <v>8.1018814766808001E-2</v>
+        <v>8.1018814766808098E-2</v>
       </c>
       <c r="D7" s="1">
         <v>6.5378189726887803E-2</v>
@@ -1130,195 +1142,195 @@
         <v>48</v>
       </c>
       <c r="G7" s="1">
-        <v>0.22128448238633899</v>
+        <v>0.22128448238633799</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+      <c r="A8" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="1">
-        <v>6.2908773988394201E-2</v>
+        <v>-0.14040289677616299</v>
       </c>
       <c r="D8" s="1">
-        <v>7.2819460877887404E-2</v>
+        <v>6.5395910146973199E-2</v>
       </c>
       <c r="E8" s="1">
-        <v>0.86390057314331603</v>
+        <v>-2.14696754675662</v>
       </c>
       <c r="F8" s="1">
         <v>48</v>
       </c>
       <c r="G8" s="1">
-        <v>0.39193908484251799</v>
+        <v>3.6876423989860699E-2</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="A9" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="1">
-        <v>6.9635722961808505E-2</v>
+        <v>-7.7494122787769001E-2</v>
       </c>
       <c r="D9" s="1">
-        <v>9.1927065415500303E-2</v>
+        <v>4.65041862174033E-2</v>
       </c>
       <c r="E9" s="1">
-        <v>0.75751056173785902</v>
+        <v>-1.66639025625543</v>
       </c>
       <c r="F9" s="1">
         <v>48</v>
       </c>
       <c r="G9" s="1">
-        <v>0.45244689645386299</v>
+        <v>0.10214920464968399</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+      <c r="A10" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C10" s="1">
-        <v>-0.119093484796503</v>
+        <v>-7.0767173814353906E-2</v>
       </c>
       <c r="D10" s="1">
-        <v>5.4450230450594099E-2</v>
+        <v>5.2950573187496297E-2</v>
       </c>
       <c r="E10" s="1">
-        <v>-2.1871989119414899</v>
+        <v>-1.3364760672895699</v>
       </c>
       <c r="F10" s="1">
         <v>48</v>
       </c>
       <c r="G10" s="1">
-        <v>3.3631929522482097E-2</v>
+        <v>0.18769466917771799</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
+      <c r="A11" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C11" s="1">
-        <v>0.16090202937235601</v>
+        <v>-0.25949638157266602</v>
       </c>
       <c r="D11" s="1">
-        <v>6.1785882124123601E-2</v>
+        <v>8.1189648183146695E-2</v>
       </c>
       <c r="E11" s="1">
-        <v>2.6041876208729202</v>
+        <v>-3.1961757118012999</v>
       </c>
       <c r="F11" s="1">
         <v>48</v>
       </c>
       <c r="G11" s="1">
-        <v>1.2220962871434E-2</v>
+        <v>2.4638523666362E-3</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+      <c r="A12" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C12" s="1">
-        <v>0.14040289677616299</v>
+        <v>2.0499132596193001E-2</v>
       </c>
       <c r="D12" s="1">
-        <v>6.5395910146973102E-2</v>
+        <v>5.6681875044213098E-2</v>
       </c>
       <c r="E12" s="1">
-        <v>2.1469675467566098</v>
+        <v>0.36165233736892499</v>
       </c>
       <c r="F12" s="1">
         <v>48</v>
       </c>
       <c r="G12" s="1">
-        <v>3.68764239898609E-2</v>
+        <v>0.71919903414918096</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
+      <c r="A13" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="1">
-        <v>-0.101138363531367</v>
+        <v>-0.24154126030753101</v>
       </c>
       <c r="D13" s="1">
-        <v>5.9760299754664299E-2</v>
+        <v>7.9140076308739205E-2</v>
       </c>
       <c r="E13" s="1">
-        <v>-1.6924005392639201</v>
+        <v>-3.0520726232969002</v>
       </c>
       <c r="F13" s="1">
         <v>48</v>
       </c>
       <c r="G13" s="1">
-        <v>9.7052037831174304E-2</v>
+        <v>3.6977862284988299E-3</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+      <c r="A14" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C14" s="1">
-        <v>8.6676987355654794E-2</v>
+        <v>-5.3725909420508498E-2</v>
       </c>
       <c r="D14" s="1">
-        <v>7.8655333692553397E-2</v>
+        <v>5.9968051180217301E-2</v>
       </c>
       <c r="E14" s="1">
-        <v>1.10198486595272</v>
+        <v>-0.89590887752963999</v>
       </c>
       <c r="F14" s="1">
         <v>48</v>
       </c>
       <c r="G14" s="1">
-        <v>0.27596325966426399</v>
+        <v>0.37477258051185502</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
+      <c r="A15" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C15" s="1">
-        <v>1.83541156082805E-2</v>
+        <v>-0.12204878116788299</v>
       </c>
       <c r="D15" s="1">
-        <v>3.3405974816938598E-2</v>
+        <v>5.7053538069678E-2</v>
       </c>
       <c r="E15" s="1">
-        <v>0.54942613436246801</v>
+        <v>-2.1391974152212501</v>
       </c>
       <c r="F15" s="1">
         <v>48</v>
       </c>
       <c r="G15" s="1">
-        <v>0.58526030548539398</v>
+        <v>3.7533818071326198E-2</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+      <c r="A16" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B16" s="1" t="s">
@@ -1331,7 +1343,7 @@
         <v>6.14293614270899E-2</v>
       </c>
       <c r="E16" s="1">
-        <v>1.63815881906038</v>
+        <v>1.63815881906039</v>
       </c>
       <c r="F16" s="1">
         <v>48</v>
@@ -1341,7 +1353,7 @@
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+      <c r="A17" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="1" t="s">
@@ -1351,20 +1363,20 @@
         <v>0.21573983771878799</v>
       </c>
       <c r="D17" s="1">
-        <v>9.8257802976814995E-2</v>
+        <v>9.8257802976815106E-2</v>
       </c>
       <c r="E17" s="1">
-        <v>2.1956509425484998</v>
+        <v>2.19565094254849</v>
       </c>
       <c r="F17" s="1">
         <v>48</v>
       </c>
       <c r="G17" s="1">
-        <v>3.2983219329057803E-2</v>
+        <v>3.2983219329058101E-2</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
+      <c r="A18" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B18" s="1" t="s">
@@ -1387,30 +1399,30 @@
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
+      <c r="A19" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>23</v>
       </c>
       <c r="C19" s="1">
-        <v>9.5389183932262298E-2</v>
+        <v>9.5389183932262006E-2</v>
       </c>
       <c r="D19" s="1">
-        <v>5.6952321271580203E-2</v>
+        <v>5.69523212715803E-2</v>
       </c>
       <c r="E19" s="1">
-        <v>1.6748954529420099</v>
+        <v>1.6748954529419999</v>
       </c>
       <c r="F19" s="1">
         <v>48</v>
       </c>
       <c r="G19" s="1">
-        <v>0.100458804351505</v>
+        <v>0.100458804351506</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
+      <c r="A20" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B20" s="1" t="s">
@@ -1420,7 +1432,7 @@
         <v>0.161635243439889</v>
       </c>
       <c r="D20" s="1">
-        <v>6.1587449596229603E-2</v>
+        <v>6.15874495962297E-2</v>
       </c>
       <c r="E20" s="1">
         <v>2.6244834702456101</v>
@@ -1429,33 +1441,38 @@
         <v>48</v>
       </c>
       <c r="G20" s="1">
-        <v>1.16034263134178E-2</v>
+        <v>1.1603426313417899E-2</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
+      <c r="A21" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C21" s="1">
-        <v>1.0760453296670999E-3</v>
+        <v>1.0760453296671899E-3</v>
       </c>
       <c r="D21" s="1">
         <v>3.78966811113184E-2</v>
       </c>
       <c r="E21" s="1">
-        <v>2.8394183820644101E-2</v>
+        <v>2.8394183820646401E-2</v>
       </c>
       <c r="F21" s="1">
         <v>48</v>
       </c>
       <c r="G21" s="1">
-        <v>0.97746549123993798</v>
+        <v>0.97746549123993598</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="G1:G1048576">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
+      <formula>0.1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>